<commit_message>
Reicher Modul-Kontext: 2-in-1 Module, Aufgaben-Sheet, Reminder
- / im Modulnamen splittet in verknuepfte Module (teilen denselben Slot)
- Zweites Excel-Sheet Aufgaben fuer woechentliche Aufgaben und Tests
- Check-in fragt Aufgaben mit Uhrzeit/Deadline-Hinweis ab
- tasks_done und linked_to im Datenmodell

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stundenplan.xlsx
+++ b/Stundenplan.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Stundenplan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Aufgaben" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +29,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
     </font>
   </fonts>
   <fills count="5">
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,6 +95,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,18 +461,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -581,31 +587,195 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Fertigungstechnik</t>
+          <t>Statistik / OR</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>VL</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fertigungstechnik</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>VL</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>GUe</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Tipp: '/' im Modulnamen = zwei Module teilen den Slot (z.B. 'Statistik / OR')</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Modul</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Beschreibung</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tage (kommagetrennt)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Uhrzeit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Deadline-Tag</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Woechentlich (ja/nein)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Online-Uebungsaufgaben</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Freitag</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mini-Test</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Montag,Mittwoch</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Operations Research</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Hausaufgaben abgeben</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Donnerstag</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>ja</t>
         </is>
       </c>
     </row>

</xml_diff>